<commit_message>
#32 Updated BOM Files
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.3/BOM/eSpark BOM IoT-Button v1.3.xlsx
+++ b/Design Files/IoT-Button-v1.3/BOM/eSpark BOM IoT-Button v1.3.xlsx
@@ -9,17 +9,20 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
+    <sheet name="100 Boards" sheetId="2" r:id="rId2"/>
+    <sheet name="500 Boards" sheetId="3" r:id="rId3"/>
+    <sheet name="5000 Boards" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="199">
   <si>
     <t>Component list</t>
   </si>
@@ -604,6 +607,18 @@
   </si>
   <si>
     <t xml:space="preserve">Multiple Lentgh Screw Required Price not Confirm </t>
+  </si>
+  <si>
+    <t>Quantity (100 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (100 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (100 Boards)</t>
   </si>
 </sst>
 </file>
@@ -1355,6 +1370,60 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20888325" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1934,9 +2003,9 @@
       <c r="P10" s="38">
         <v>5.1999999999999998E-3</v>
       </c>
-      <c r="Q10" s="38">
-        <f>P11*N11</f>
-        <v>0.18</v>
+      <c r="Q10" s="60">
+        <f>P10*N10</f>
+        <v>0.52</v>
       </c>
       <c r="R10" s="37"/>
       <c r="S10" s="49"/>
@@ -1990,9 +2059,9 @@
       <c r="P11" s="38">
         <v>1.8E-3</v>
       </c>
-      <c r="Q11" s="38">
-        <f>P12*N12</f>
-        <v>2.0579999999999998</v>
+      <c r="Q11" s="60">
+        <f t="shared" ref="Q11:Q38" si="2">P11*N11</f>
+        <v>0.18</v>
       </c>
       <c r="R11" s="50"/>
       <c r="S11" s="50"/>
@@ -2046,8 +2115,8 @@
       <c r="P12" s="38">
         <v>0.13719999999999999</v>
       </c>
-      <c r="Q12" s="38">
-        <f>P12*N12</f>
+      <c r="Q12" s="60">
+        <f t="shared" si="2"/>
         <v>2.0579999999999998</v>
       </c>
       <c r="R12" s="37"/>
@@ -2090,7 +2159,7 @@
         <v>1</v>
       </c>
       <c r="M13" s="50">
-        <f t="shared" ref="M13" si="2">L13*5</f>
+        <f t="shared" ref="M13" si="3">L13*5</f>
         <v>5</v>
       </c>
       <c r="N13" s="37">
@@ -2102,8 +2171,8 @@
       <c r="P13" s="38">
         <v>3.4099999999999998E-2</v>
       </c>
-      <c r="Q13" s="51">
-        <f t="shared" ref="Q13" si="3">P13*N13</f>
+      <c r="Q13" s="60">
+        <f t="shared" si="2"/>
         <v>0.34099999999999997</v>
       </c>
       <c r="R13" s="50"/>
@@ -2158,8 +2227,8 @@
       <c r="P14" s="51">
         <v>0.82730000000000004</v>
       </c>
-      <c r="Q14" s="38">
-        <f>P14*N14</f>
+      <c r="Q14" s="60">
+        <f t="shared" si="2"/>
         <v>4.9638</v>
       </c>
       <c r="R14" s="37"/>
@@ -2214,8 +2283,8 @@
       <c r="P15" s="38">
         <v>9.3299999999999994E-2</v>
       </c>
-      <c r="Q15" s="51">
-        <f t="shared" ref="Q15" si="5">P15*N15</f>
+      <c r="Q15" s="60">
+        <f t="shared" si="2"/>
         <v>0.93299999999999994</v>
       </c>
       <c r="R15" s="50"/>
@@ -2270,8 +2339,8 @@
       <c r="P16" s="51">
         <v>2.7199999999999998E-2</v>
       </c>
-      <c r="Q16" s="38">
-        <f>P16*N16</f>
+      <c r="Q16" s="60">
+        <f t="shared" si="2"/>
         <v>0.54399999999999993</v>
       </c>
       <c r="R16" s="37"/>
@@ -2314,7 +2383,7 @@
         <v>1</v>
       </c>
       <c r="M17" s="50">
-        <f t="shared" ref="M17" si="6">L17*5</f>
+        <f t="shared" ref="M17" si="5">L17*5</f>
         <v>5</v>
       </c>
       <c r="N17" s="50">
@@ -2326,8 +2395,8 @@
       <c r="P17" s="38">
         <v>0.1318</v>
       </c>
-      <c r="Q17" s="51">
-        <f t="shared" ref="Q17" si="7">P17*N17</f>
+      <c r="Q17" s="60">
+        <f t="shared" si="2"/>
         <v>1.3180000000000001</v>
       </c>
       <c r="R17" s="50"/>
@@ -2382,8 +2451,8 @@
       <c r="P18" s="51">
         <v>2.1700000000000001E-2</v>
       </c>
-      <c r="Q18" s="38">
-        <f>P18*N18</f>
+      <c r="Q18" s="60">
+        <f t="shared" si="2"/>
         <v>0.434</v>
       </c>
       <c r="R18" s="37"/>
@@ -2426,7 +2495,7 @@
         <v>1</v>
       </c>
       <c r="M19" s="50">
-        <f t="shared" ref="M19" si="8">L19*5</f>
+        <f t="shared" ref="M19" si="6">L19*5</f>
         <v>5</v>
       </c>
       <c r="N19" s="37">
@@ -2438,8 +2507,8 @@
       <c r="P19" s="38">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="Q19" s="51">
-        <f t="shared" ref="Q19" si="9">P19*N19</f>
+      <c r="Q19" s="60">
+        <f t="shared" si="2"/>
         <v>0.81600000000000006</v>
       </c>
       <c r="R19" s="50"/>
@@ -2494,8 +2563,8 @@
       <c r="P20" s="51">
         <v>2.0799999999999999E-2</v>
       </c>
-      <c r="Q20" s="38">
-        <f>P20*N20</f>
+      <c r="Q20" s="60">
+        <f t="shared" si="2"/>
         <v>0.41599999999999998</v>
       </c>
       <c r="R20" s="37"/>
@@ -2538,7 +2607,7 @@
         <v>6</v>
       </c>
       <c r="M21" s="50">
-        <f t="shared" ref="M21" si="10">L21*5</f>
+        <f t="shared" ref="M21" si="7">L21*5</f>
         <v>30</v>
       </c>
       <c r="N21" s="37">
@@ -2550,8 +2619,8 @@
       <c r="P21" s="38">
         <v>6.1699999999999998E-2</v>
       </c>
-      <c r="Q21" s="51">
-        <f t="shared" ref="Q21" si="11">P21*N21</f>
+      <c r="Q21" s="60">
+        <f t="shared" si="2"/>
         <v>2.468</v>
       </c>
       <c r="R21" s="50"/>
@@ -2606,8 +2675,8 @@
       <c r="P22" s="38">
         <v>3.4099999999999998E-2</v>
       </c>
-      <c r="Q22" s="38">
-        <f>P22*N22</f>
+      <c r="Q22" s="60">
+        <f t="shared" si="2"/>
         <v>0.68199999999999994</v>
       </c>
       <c r="R22" s="37"/>
@@ -2650,7 +2719,7 @@
         <v>1</v>
       </c>
       <c r="M23" s="50">
-        <f t="shared" ref="M23" si="12">L23*5</f>
+        <f t="shared" ref="M23" si="8">L23*5</f>
         <v>5</v>
       </c>
       <c r="N23" s="62">
@@ -2662,8 +2731,8 @@
       <c r="P23" s="64">
         <v>2.9399999999999999E-2</v>
       </c>
-      <c r="Q23" s="51">
-        <f t="shared" ref="Q23" si="13">P23*N23</f>
+      <c r="Q23" s="60">
+        <f t="shared" si="2"/>
         <v>0.58799999999999997</v>
       </c>
       <c r="R23" s="50"/>
@@ -2718,8 +2787,8 @@
       <c r="P24" s="38">
         <v>1E-3</v>
       </c>
-      <c r="Q24" s="38">
-        <f>P24*N24</f>
+      <c r="Q24" s="60">
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="R24" s="37"/>
@@ -2762,7 +2831,7 @@
         <v>1</v>
       </c>
       <c r="M25" s="50">
-        <f t="shared" ref="M25" si="14">L25*5</f>
+        <f t="shared" ref="M25" si="9">L25*5</f>
         <v>5</v>
       </c>
       <c r="N25" s="37">
@@ -2774,8 +2843,8 @@
       <c r="P25" s="38">
         <v>6.9999999999999999E-4</v>
       </c>
-      <c r="Q25" s="51">
-        <f t="shared" ref="Q25" si="15">P25*N25</f>
+      <c r="Q25" s="60">
+        <f t="shared" si="2"/>
         <v>6.9999999999999993E-2</v>
       </c>
       <c r="R25" s="50"/>
@@ -2830,8 +2899,8 @@
       <c r="P26" s="38">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="Q26" s="38">
-        <f>P26*N26</f>
+      <c r="Q26" s="60">
+        <f t="shared" si="2"/>
         <v>0.11</v>
       </c>
       <c r="R26" s="37"/>
@@ -2874,7 +2943,7 @@
         <v>1</v>
       </c>
       <c r="M27" s="50">
-        <f t="shared" ref="M27" si="16">L27*5</f>
+        <f t="shared" ref="M27" si="10">L27*5</f>
         <v>5</v>
       </c>
       <c r="N27" s="37">
@@ -2886,8 +2955,8 @@
       <c r="P27" s="38">
         <v>1E-3</v>
       </c>
-      <c r="Q27" s="51">
-        <f t="shared" ref="Q27" si="17">P27*N27</f>
+      <c r="Q27" s="60">
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="R27" s="50"/>
@@ -2942,8 +3011,8 @@
       <c r="P28" s="38">
         <v>1E-3</v>
       </c>
-      <c r="Q28" s="51">
-        <f>P28*N28</f>
+      <c r="Q28" s="60">
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="R28" s="37"/>
@@ -2986,7 +3055,7 @@
         <v>2</v>
       </c>
       <c r="M29" s="50">
-        <f t="shared" ref="M29" si="18">L29*5</f>
+        <f t="shared" ref="M29" si="11">L29*5</f>
         <v>10</v>
       </c>
       <c r="N29" s="50">
@@ -2998,8 +3067,8 @@
       <c r="P29" s="51">
         <v>3.9899999999999998E-2</v>
       </c>
-      <c r="Q29" s="51">
-        <f t="shared" ref="Q29" si="19">P29*N29</f>
+      <c r="Q29" s="60">
+        <f t="shared" si="2"/>
         <v>0.79799999999999993</v>
       </c>
       <c r="R29" s="50"/>
@@ -3054,8 +3123,8 @@
       <c r="P30" s="38">
         <v>5.6800000000000003E-2</v>
       </c>
-      <c r="Q30" s="38">
-        <f>P30*N30</f>
+      <c r="Q30" s="60">
+        <f t="shared" si="2"/>
         <v>0.56800000000000006</v>
       </c>
       <c r="R30" s="37"/>
@@ -3098,7 +3167,7 @@
         <v>1</v>
       </c>
       <c r="M31" s="50">
-        <f t="shared" ref="M31" si="20">L31*5</f>
+        <f t="shared" ref="M31" si="12">L31*5</f>
         <v>5</v>
       </c>
       <c r="N31" s="37">
@@ -3110,8 +3179,8 @@
       <c r="P31" s="38">
         <v>0.13020000000000001</v>
       </c>
-      <c r="Q31" s="51">
-        <f t="shared" ref="Q31" si="21">P31*N31</f>
+      <c r="Q31" s="60">
+        <f t="shared" si="2"/>
         <v>1.302</v>
       </c>
       <c r="R31" s="50"/>
@@ -3166,8 +3235,8 @@
       <c r="P32" s="51">
         <v>0.17599999999999999</v>
       </c>
-      <c r="Q32" s="38">
-        <f>P32*N32</f>
+      <c r="Q32" s="60">
+        <f t="shared" si="2"/>
         <v>1.7599999999999998</v>
       </c>
       <c r="R32" s="37"/>
@@ -3210,7 +3279,7 @@
         <v>1</v>
       </c>
       <c r="M33" s="50">
-        <f t="shared" ref="M33" si="22">L33*5</f>
+        <f t="shared" ref="M33" si="13">L33*5</f>
         <v>5</v>
       </c>
       <c r="N33" s="50">
@@ -3222,8 +3291,8 @@
       <c r="P33" s="51">
         <v>3.3075000000000001</v>
       </c>
-      <c r="Q33" s="51">
-        <f t="shared" ref="Q33" si="23">P33*N33</f>
+      <c r="Q33" s="60">
+        <f t="shared" si="2"/>
         <v>19.844999999999999</v>
       </c>
       <c r="R33" s="50"/>
@@ -3278,8 +3347,8 @@
       <c r="P34" s="51">
         <v>0.54569999999999996</v>
       </c>
-      <c r="Q34" s="38">
-        <f>P34*N34</f>
+      <c r="Q34" s="60">
+        <f t="shared" si="2"/>
         <v>3.2741999999999996</v>
       </c>
       <c r="R34" s="37"/>
@@ -3288,7 +3357,7 @@
     <row r="35" spans="1:26" ht="48" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="45">
-        <f t="shared" ref="B35:B38" si="24">ROW(B35) - ROW($B$9)</f>
+        <f t="shared" ref="B35:B38" si="14">ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
       <c r="C35" s="52" t="s">
@@ -3334,8 +3403,8 @@
       <c r="P35" s="38">
         <v>4.67</v>
       </c>
-      <c r="Q35" s="38">
-        <f>P35*N35</f>
+      <c r="Q35" s="60">
+        <f t="shared" si="2"/>
         <v>23.35</v>
       </c>
       <c r="R35" s="37"/>
@@ -3344,7 +3413,7 @@
     <row r="36" spans="1:26" ht="48" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="45">
-        <f t="shared" si="24"/>
+        <f t="shared" si="14"/>
         <v>27</v>
       </c>
       <c r="C36" s="52" t="s">
@@ -3391,7 +3460,7 @@
         <v>0.35</v>
       </c>
       <c r="Q36" s="60">
-        <f>P36*N36</f>
+        <f t="shared" si="2"/>
         <v>0.35</v>
       </c>
       <c r="R36" s="37"/>
@@ -3400,7 +3469,7 @@
     <row r="37" spans="1:26" ht="24" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="45">
-        <f t="shared" si="24"/>
+        <f t="shared" si="14"/>
         <v>28</v>
       </c>
       <c r="C37" s="52" t="s">
@@ -3447,7 +3516,7 @@
         <v>16.989999999999998</v>
       </c>
       <c r="Q37" s="60">
-        <f>P37*N37</f>
+        <f t="shared" si="2"/>
         <v>16.989999999999998</v>
       </c>
       <c r="R37" s="37"/>
@@ -3456,7 +3525,7 @@
     <row r="38" spans="1:26" s="67" customFormat="1" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="66"/>
       <c r="B38" s="45">
-        <f t="shared" si="24"/>
+        <f t="shared" si="14"/>
         <v>29</v>
       </c>
       <c r="C38" s="52" t="s">
@@ -3503,7 +3572,8 @@
         <v>3</v>
       </c>
       <c r="Q38" s="60">
-        <v>3</v>
+        <f t="shared" si="2"/>
+        <v>300</v>
       </c>
       <c r="R38" s="65" t="s">
         <v>194</v>
@@ -3537,7 +3607,7 @@
       <c r="P39" s="77"/>
       <c r="Q39" s="47">
         <f>SUM(Q10:Q38)</f>
-        <v>89.516999999999996</v>
+        <v>384.97899999999998</v>
       </c>
       <c r="R39" s="72"/>
       <c r="S39" s="73"/>
@@ -3563,7 +3633,7 @@
       <c r="P40" s="77"/>
       <c r="Q40" s="48">
         <f>Q39/5</f>
-        <v>17.903399999999998</v>
+        <v>76.995800000000003</v>
       </c>
       <c r="R40" s="74"/>
       <c r="S40" s="75"/>
@@ -3611,4 +3681,2008 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId30"/>
   <drawing r:id="rId31"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S40"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="68"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="69"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="54" t="s">
+        <v>168</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="70"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="56" t="s">
+        <v>169</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="71"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="57" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="71"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="71"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="71"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="71"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>135</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="B10" s="45">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I10" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="L10" s="37">
+        <v>6</v>
+      </c>
+      <c r="M10" s="37">
+        <f>L10*100</f>
+        <v>600</v>
+      </c>
+      <c r="N10" s="37">
+        <v>700</v>
+      </c>
+      <c r="O10" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P10" s="38">
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="Q10" s="60">
+        <f>P10*N10</f>
+        <v>4.13</v>
+      </c>
+      <c r="R10" s="37"/>
+      <c r="S10" s="49"/>
+    </row>
+    <row r="11" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="B11" s="46">
+        <f t="shared" ref="B11:B33" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" s="50" t="s">
+        <v>98</v>
+      </c>
+      <c r="H11" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I11" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="J11" s="50" t="s">
+        <v>137</v>
+      </c>
+      <c r="K11" s="50" t="s">
+        <v>160</v>
+      </c>
+      <c r="L11" s="50">
+        <v>15</v>
+      </c>
+      <c r="M11" s="37">
+        <f t="shared" ref="M11:M38" si="1">L11*100</f>
+        <v>1500</v>
+      </c>
+      <c r="N11" s="37">
+        <v>1600</v>
+      </c>
+      <c r="O11" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P11" s="38">
+        <v>1.5E-3</v>
+      </c>
+      <c r="Q11" s="60">
+        <f t="shared" ref="Q11:Q38" si="2">P11*N11</f>
+        <v>2.4</v>
+      </c>
+      <c r="R11" s="50"/>
+      <c r="S11" s="50"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="45">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J12" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="K12" s="37" t="s">
+        <v>161</v>
+      </c>
+      <c r="L12" s="37">
+        <v>2</v>
+      </c>
+      <c r="M12" s="37">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N12" s="37">
+        <v>205</v>
+      </c>
+      <c r="O12" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P12" s="38">
+        <v>0.10199999999999999</v>
+      </c>
+      <c r="Q12" s="60">
+        <f t="shared" si="2"/>
+        <v>20.91</v>
+      </c>
+      <c r="R12" s="37"/>
+      <c r="S12" s="58"/>
+    </row>
+    <row r="13" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="46">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" s="50" t="s">
+        <v>100</v>
+      </c>
+      <c r="H13" s="50" t="s">
+        <v>118</v>
+      </c>
+      <c r="I13" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J13" s="50" t="s">
+        <v>139</v>
+      </c>
+      <c r="K13" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L13" s="50">
+        <v>1</v>
+      </c>
+      <c r="M13" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N13" s="37">
+        <v>110</v>
+      </c>
+      <c r="O13" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P13" s="38">
+        <v>2.7400000000000001E-2</v>
+      </c>
+      <c r="Q13" s="60">
+        <f t="shared" si="2"/>
+        <v>3.0140000000000002</v>
+      </c>
+      <c r="R13" s="50"/>
+      <c r="S13" s="58"/>
+    </row>
+    <row r="14" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="45">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="K14" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="L14" s="37">
+        <v>1</v>
+      </c>
+      <c r="M14" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N14" s="50">
+        <v>101</v>
+      </c>
+      <c r="O14" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P14" s="51">
+        <v>0.5696</v>
+      </c>
+      <c r="Q14" s="60">
+        <f t="shared" si="2"/>
+        <v>57.529600000000002</v>
+      </c>
+      <c r="R14" s="37"/>
+      <c r="S14" s="58"/>
+    </row>
+    <row r="15" spans="1:19" ht="36" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="46">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="53" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="50" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="50" t="s">
+        <v>102</v>
+      </c>
+      <c r="H15" s="50" t="s">
+        <v>120</v>
+      </c>
+      <c r="I15" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J15" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="K15" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L15" s="50">
+        <v>1</v>
+      </c>
+      <c r="M15" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N15" s="37">
+        <v>105</v>
+      </c>
+      <c r="O15" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P15" s="38">
+        <v>7.5999999999999998E-2</v>
+      </c>
+      <c r="Q15" s="60">
+        <f t="shared" si="2"/>
+        <v>7.9799999999999995</v>
+      </c>
+      <c r="R15" s="50"/>
+      <c r="S15" s="58"/>
+    </row>
+    <row r="16" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="45">
+        <f>ROW(B16) - ROW($B$9)</f>
+        <v>7</v>
+      </c>
+      <c r="C16" s="52" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="H16" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="I16" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J16" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="K16" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L16" s="37">
+        <v>1</v>
+      </c>
+      <c r="M16" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N16" s="50">
+        <v>120</v>
+      </c>
+      <c r="O16" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P16" s="51">
+        <v>2.64E-2</v>
+      </c>
+      <c r="Q16" s="60">
+        <f t="shared" si="2"/>
+        <v>3.1680000000000001</v>
+      </c>
+      <c r="R16" s="37"/>
+      <c r="S16" s="58"/>
+    </row>
+    <row r="17" spans="1:19" ht="48" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="46">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="C17" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G17" s="50" t="s">
+        <v>82</v>
+      </c>
+      <c r="H17" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="I17" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J17" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="K17" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L17" s="50">
+        <v>1</v>
+      </c>
+      <c r="M17" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N17" s="50">
+        <v>105</v>
+      </c>
+      <c r="O17" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P17" s="38">
+        <v>0.105</v>
+      </c>
+      <c r="Q17" s="60">
+        <f t="shared" si="2"/>
+        <v>11.025</v>
+      </c>
+      <c r="R17" s="50"/>
+      <c r="S17" s="58"/>
+    </row>
+    <row r="18" spans="1:19" ht="48" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="45">
+        <f>ROW(B18) - ROW($B$9)</f>
+        <v>9</v>
+      </c>
+      <c r="C18" s="52" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G18" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J18" s="37" t="s">
+        <v>144</v>
+      </c>
+      <c r="K18" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L18" s="37">
+        <v>1</v>
+      </c>
+      <c r="M18" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N18" s="50">
+        <v>120</v>
+      </c>
+      <c r="O18" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P18" s="51">
+        <v>2.1700000000000001E-2</v>
+      </c>
+      <c r="Q18" s="60">
+        <f t="shared" si="2"/>
+        <v>2.6040000000000001</v>
+      </c>
+      <c r="R18" s="37"/>
+      <c r="S18" s="58"/>
+    </row>
+    <row r="19" spans="1:19" ht="36" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="46">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C19" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="50" t="s">
+        <v>59</v>
+      </c>
+      <c r="F19" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G19" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="H19" s="50" t="s">
+        <v>124</v>
+      </c>
+      <c r="I19" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J19" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="K19" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L19" s="50">
+        <v>1</v>
+      </c>
+      <c r="M19" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N19" s="37">
+        <v>108</v>
+      </c>
+      <c r="O19" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P19" s="38">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="Q19" s="60">
+        <f t="shared" si="2"/>
+        <v>7.3440000000000003</v>
+      </c>
+      <c r="R19" s="50"/>
+      <c r="S19" s="58"/>
+    </row>
+    <row r="20" spans="1:19" ht="48" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="45">
+        <f>ROW(B20) - ROW($B$9)</f>
+        <v>11</v>
+      </c>
+      <c r="C20" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="G20" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="H20" s="37" t="s">
+        <v>125</v>
+      </c>
+      <c r="I20" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J20" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="K20" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L20" s="37">
+        <v>1</v>
+      </c>
+      <c r="M20" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N20" s="50">
+        <v>120</v>
+      </c>
+      <c r="O20" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P20" s="51">
+        <v>2.0799999999999999E-2</v>
+      </c>
+      <c r="Q20" s="60">
+        <f t="shared" si="2"/>
+        <v>2.496</v>
+      </c>
+      <c r="R20" s="37"/>
+      <c r="S20" s="58"/>
+    </row>
+    <row r="21" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="46">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C21" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="50" t="s">
+        <v>35</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G21" s="50" t="s">
+        <v>85</v>
+      </c>
+      <c r="H21" s="50" t="s">
+        <v>126</v>
+      </c>
+      <c r="I21" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J21" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="K21" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L21" s="50">
+        <v>6</v>
+      </c>
+      <c r="M21" s="37">
+        <f t="shared" si="1"/>
+        <v>600</v>
+      </c>
+      <c r="N21" s="37">
+        <v>610</v>
+      </c>
+      <c r="O21" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P21" s="38">
+        <v>4.4400000000000002E-2</v>
+      </c>
+      <c r="Q21" s="60">
+        <f t="shared" si="2"/>
+        <v>27.084</v>
+      </c>
+      <c r="R21" s="50"/>
+      <c r="S21" s="58"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="45">
+        <f>ROW(B22) - ROW($B$9)</f>
+        <v>13</v>
+      </c>
+      <c r="C22" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="F22" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="G22" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="H22" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="I22" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J22" s="37" t="s">
+        <v>147</v>
+      </c>
+      <c r="K22" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L22" s="37">
+        <v>1</v>
+      </c>
+      <c r="M22" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N22" s="37">
+        <v>20</v>
+      </c>
+      <c r="O22" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P22" s="38">
+        <v>3.4099999999999998E-2</v>
+      </c>
+      <c r="Q22" s="60">
+        <f t="shared" si="2"/>
+        <v>0.68199999999999994</v>
+      </c>
+      <c r="R22" s="37"/>
+      <c r="S22" s="58"/>
+    </row>
+    <row r="23" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="46">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C23" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="E23" s="50" t="s">
+        <v>63</v>
+      </c>
+      <c r="F23" s="50" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" s="50" t="s">
+        <v>107</v>
+      </c>
+      <c r="H23" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="I23" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J23" s="50" t="s">
+        <v>148</v>
+      </c>
+      <c r="K23" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L23" s="50">
+        <v>1</v>
+      </c>
+      <c r="M23" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N23" s="62">
+        <v>20</v>
+      </c>
+      <c r="O23" s="63" t="s">
+        <v>179</v>
+      </c>
+      <c r="P23" s="64">
+        <v>2.9399999999999999E-2</v>
+      </c>
+      <c r="Q23" s="60">
+        <f t="shared" si="2"/>
+        <v>0.58799999999999997</v>
+      </c>
+      <c r="R23" s="50"/>
+      <c r="S23" s="58"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="B24" s="45">
+        <f>ROW(B24) - ROW($B$9)</f>
+        <v>15</v>
+      </c>
+      <c r="C24" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="F24" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G24" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="H24" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I24" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J24" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="K24" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="L24" s="37">
+        <v>7</v>
+      </c>
+      <c r="M24" s="37">
+        <f t="shared" si="1"/>
+        <v>700</v>
+      </c>
+      <c r="N24" s="37">
+        <v>100</v>
+      </c>
+      <c r="O24" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P24" s="38">
+        <v>1E-3</v>
+      </c>
+      <c r="Q24" s="60">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="R24" s="37"/>
+      <c r="S24" s="58"/>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="46">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C25" s="53" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="F25" s="50" t="s">
+        <v>89</v>
+      </c>
+      <c r="G25" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="H25" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I25" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J25" s="50" t="s">
+        <v>150</v>
+      </c>
+      <c r="K25" s="50" t="s">
+        <v>163</v>
+      </c>
+      <c r="L25" s="50">
+        <v>1</v>
+      </c>
+      <c r="M25" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N25" s="37">
+        <v>100</v>
+      </c>
+      <c r="O25" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P25" s="38">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q25" s="60">
+        <f t="shared" si="2"/>
+        <v>6.9999999999999993E-2</v>
+      </c>
+      <c r="R25" s="50"/>
+      <c r="S25" s="58"/>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="45">
+        <f>ROW(B26) - ROW($B$9)</f>
+        <v>17</v>
+      </c>
+      <c r="C26" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="F26" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G26" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="H26" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I26" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J26" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="K26" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="L26" s="37">
+        <v>2</v>
+      </c>
+      <c r="M26" s="37">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N26" s="37">
+        <v>100</v>
+      </c>
+      <c r="O26" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P26" s="38">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q26" s="60">
+        <f t="shared" si="2"/>
+        <v>0.11</v>
+      </c>
+      <c r="R26" s="37"/>
+      <c r="S26" s="58"/>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A27" s="1"/>
+      <c r="B27" s="46">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="C27" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="50" t="s">
+        <v>41</v>
+      </c>
+      <c r="E27" s="50" t="s">
+        <v>67</v>
+      </c>
+      <c r="F27" s="50" t="s">
+        <v>88</v>
+      </c>
+      <c r="G27" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="H27" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I27" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J27" s="50" t="s">
+        <v>152</v>
+      </c>
+      <c r="K27" s="50" t="s">
+        <v>165</v>
+      </c>
+      <c r="L27" s="50">
+        <v>1</v>
+      </c>
+      <c r="M27" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N27" s="37">
+        <v>100</v>
+      </c>
+      <c r="O27" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P27" s="38">
+        <v>1E-3</v>
+      </c>
+      <c r="Q27" s="60">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="R27" s="50"/>
+      <c r="S27" s="58"/>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="B28" s="45">
+        <f>ROW(B28) - ROW($B$9)</f>
+        <v>19</v>
+      </c>
+      <c r="C28" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="F28" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G28" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="H28" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I28" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J28" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="K28" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="L28" s="37">
+        <v>1</v>
+      </c>
+      <c r="M28" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N28" s="37">
+        <v>100</v>
+      </c>
+      <c r="O28" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P28" s="38">
+        <v>1E-3</v>
+      </c>
+      <c r="Q28" s="60">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="R28" s="37"/>
+      <c r="S28" s="58"/>
+    </row>
+    <row r="29" spans="1:19" ht="36" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="B29" s="46">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="C29" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" s="50" t="s">
+        <v>69</v>
+      </c>
+      <c r="F29" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G29" s="50" t="s">
+        <v>90</v>
+      </c>
+      <c r="H29" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="I29" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J29" s="50" t="s">
+        <v>154</v>
+      </c>
+      <c r="K29" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L29" s="50">
+        <v>2</v>
+      </c>
+      <c r="M29" s="37">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N29" s="50">
+        <v>20</v>
+      </c>
+      <c r="O29" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P29" s="51">
+        <v>3.9899999999999998E-2</v>
+      </c>
+      <c r="Q29" s="60">
+        <f t="shared" si="2"/>
+        <v>0.79799999999999993</v>
+      </c>
+      <c r="R29" s="50"/>
+      <c r="S29" s="58"/>
+    </row>
+    <row r="30" spans="1:19" ht="48" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="B30" s="45">
+        <f>ROW(B30) - ROW($B$9)</f>
+        <v>21</v>
+      </c>
+      <c r="C30" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G30" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="H30" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="I30" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J30" s="37" t="s">
+        <v>155</v>
+      </c>
+      <c r="K30" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L30" s="37">
+        <v>1</v>
+      </c>
+      <c r="M30" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N30" s="37">
+        <v>10</v>
+      </c>
+      <c r="O30" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P30" s="38">
+        <v>5.6800000000000003E-2</v>
+      </c>
+      <c r="Q30" s="60">
+        <f t="shared" si="2"/>
+        <v>0.56800000000000006</v>
+      </c>
+      <c r="R30" s="37"/>
+      <c r="S30" s="58"/>
+    </row>
+    <row r="31" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="46">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C31" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="F31" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G31" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="H31" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="I31" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J31" s="37" t="s">
+        <v>191</v>
+      </c>
+      <c r="K31" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L31" s="50">
+        <v>1</v>
+      </c>
+      <c r="M31" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N31" s="37">
+        <v>10</v>
+      </c>
+      <c r="O31" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P31" s="38">
+        <v>0.13020000000000001</v>
+      </c>
+      <c r="Q31" s="60">
+        <f t="shared" si="2"/>
+        <v>1.302</v>
+      </c>
+      <c r="R31" s="50"/>
+      <c r="S31" s="58"/>
+    </row>
+    <row r="32" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="B32" s="45">
+        <f>ROW(B32) - ROW($B$9)</f>
+        <v>23</v>
+      </c>
+      <c r="C32" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="F32" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="G32" s="37" t="s">
+        <v>113</v>
+      </c>
+      <c r="H32" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="I32" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J32" s="37" t="s">
+        <v>156</v>
+      </c>
+      <c r="K32" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L32" s="37">
+        <v>1</v>
+      </c>
+      <c r="M32" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N32" s="50">
+        <v>10</v>
+      </c>
+      <c r="O32" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P32" s="51">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="Q32" s="60">
+        <f t="shared" si="2"/>
+        <v>1.7599999999999998</v>
+      </c>
+      <c r="R32" s="37"/>
+      <c r="S32" s="58"/>
+    </row>
+    <row r="33" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="B33" s="46">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="C33" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="E33" s="50" t="s">
+        <v>73</v>
+      </c>
+      <c r="F33" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="G33" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="H33" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="I33" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J33" s="50" t="s">
+        <v>157</v>
+      </c>
+      <c r="K33" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L33" s="50">
+        <v>1</v>
+      </c>
+      <c r="M33" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N33" s="50">
+        <v>6</v>
+      </c>
+      <c r="O33" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P33" s="51">
+        <v>3.3075000000000001</v>
+      </c>
+      <c r="Q33" s="60">
+        <f t="shared" si="2"/>
+        <v>19.844999999999999</v>
+      </c>
+      <c r="R33" s="50"/>
+      <c r="S33" s="58"/>
+    </row>
+    <row r="34" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="B34" s="45">
+        <f>ROW(B34) - ROW($B$9)</f>
+        <v>25</v>
+      </c>
+      <c r="C34" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>74</v>
+      </c>
+      <c r="F34" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="G34" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="H34" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="I34" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J34" s="37" t="s">
+        <v>158</v>
+      </c>
+      <c r="K34" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L34" s="37">
+        <v>1</v>
+      </c>
+      <c r="M34" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N34" s="50">
+        <v>6</v>
+      </c>
+      <c r="O34" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P34" s="51">
+        <v>0.54569999999999996</v>
+      </c>
+      <c r="Q34" s="60">
+        <f t="shared" si="2"/>
+        <v>3.2741999999999996</v>
+      </c>
+      <c r="R34" s="37"/>
+      <c r="S34" s="58"/>
+    </row>
+    <row r="35" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="A35" s="1"/>
+      <c r="B35" s="45">
+        <f t="shared" ref="B35:B38" si="3">ROW(B35) - ROW($B$9)</f>
+        <v>26</v>
+      </c>
+      <c r="C35" s="52" t="s">
+        <v>181</v>
+      </c>
+      <c r="D35" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E35" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="F35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K35" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L35" s="37">
+        <v>1</v>
+      </c>
+      <c r="M35" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N35" s="37">
+        <v>5</v>
+      </c>
+      <c r="O35" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="P35" s="38">
+        <v>4.67</v>
+      </c>
+      <c r="Q35" s="60">
+        <f t="shared" si="2"/>
+        <v>23.35</v>
+      </c>
+      <c r="R35" s="37"/>
+      <c r="S35" s="58"/>
+    </row>
+    <row r="36" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="B36" s="45">
+        <f t="shared" si="3"/>
+        <v>27</v>
+      </c>
+      <c r="C36" s="52" t="s">
+        <v>185</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="F36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K36" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L36" s="37">
+        <v>1</v>
+      </c>
+      <c r="M36" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N36" s="37">
+        <v>1</v>
+      </c>
+      <c r="O36" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="P36" s="38">
+        <v>0.35</v>
+      </c>
+      <c r="Q36" s="60">
+        <f t="shared" si="2"/>
+        <v>0.35</v>
+      </c>
+      <c r="R36" s="37"/>
+      <c r="S36" s="58"/>
+    </row>
+    <row r="37" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1"/>
+      <c r="B37" s="45">
+        <f t="shared" si="3"/>
+        <v>28</v>
+      </c>
+      <c r="C37" s="52" t="s">
+        <v>187</v>
+      </c>
+      <c r="D37" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E37" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="F37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K37" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L37" s="37">
+        <v>1</v>
+      </c>
+      <c r="M37" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N37" s="37">
+        <v>1</v>
+      </c>
+      <c r="O37" s="59" t="s">
+        <v>188</v>
+      </c>
+      <c r="P37" s="38">
+        <v>16.989999999999998</v>
+      </c>
+      <c r="Q37" s="60">
+        <f t="shared" si="2"/>
+        <v>16.989999999999998</v>
+      </c>
+      <c r="R37" s="37"/>
+      <c r="S37" s="58"/>
+    </row>
+    <row r="38" spans="1:19" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="66"/>
+      <c r="B38" s="45">
+        <f t="shared" si="3"/>
+        <v>29</v>
+      </c>
+      <c r="C38" s="52" t="s">
+        <v>192</v>
+      </c>
+      <c r="D38" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E38" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="F38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K38" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L38" s="37">
+        <v>4</v>
+      </c>
+      <c r="M38" s="37">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+      <c r="N38" s="37">
+        <v>100</v>
+      </c>
+      <c r="O38" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="P38" s="38">
+        <v>3</v>
+      </c>
+      <c r="Q38" s="60">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="R38" s="65" t="s">
+        <v>194</v>
+      </c>
+      <c r="S38" s="58"/>
+    </row>
+    <row r="39" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1"/>
+      <c r="B39" s="39"/>
+      <c r="C39" s="40"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="42"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="44"/>
+      <c r="H39" s="43"/>
+      <c r="I39" s="44"/>
+      <c r="J39" s="43"/>
+      <c r="K39" s="44"/>
+      <c r="L39" s="44"/>
+      <c r="M39" s="44"/>
+      <c r="N39" s="76" t="s">
+        <v>5</v>
+      </c>
+      <c r="O39" s="77"/>
+      <c r="P39" s="77"/>
+      <c r="Q39" s="47">
+        <f>SUM(Q10:Q38)</f>
+        <v>519.67179999999996</v>
+      </c>
+      <c r="R39" s="72"/>
+      <c r="S39" s="73"/>
+    </row>
+    <row r="40" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="1"/>
+      <c r="B40" s="25"/>
+      <c r="C40" s="36"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="76" t="s">
+        <v>6</v>
+      </c>
+      <c r="O40" s="77"/>
+      <c r="P40" s="77"/>
+      <c r="Q40" s="48">
+        <f>Q39/100</f>
+        <v>5.1967179999999997</v>
+      </c>
+      <c r="R40" s="74"/>
+      <c r="S40" s="75"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N39:P39"/>
+    <mergeCell ref="R39:S40"/>
+    <mergeCell ref="N40:P40"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O11" r:id="rId1"/>
+    <hyperlink ref="O35" r:id="rId2"/>
+    <hyperlink ref="O36" r:id="rId3"/>
+    <hyperlink ref="O37" r:id="rId4"/>
+    <hyperlink ref="O10" r:id="rId5"/>
+    <hyperlink ref="O12" r:id="rId6"/>
+    <hyperlink ref="O13" r:id="rId7"/>
+    <hyperlink ref="O15" r:id="rId8"/>
+    <hyperlink ref="O16" r:id="rId9"/>
+    <hyperlink ref="O18" r:id="rId10"/>
+    <hyperlink ref="O19" r:id="rId11"/>
+    <hyperlink ref="O14" r:id="rId12"/>
+    <hyperlink ref="O17" r:id="rId13"/>
+    <hyperlink ref="O20" r:id="rId14"/>
+    <hyperlink ref="O24" r:id="rId15"/>
+    <hyperlink ref="O21" r:id="rId16"/>
+    <hyperlink ref="O23" r:id="rId17"/>
+    <hyperlink ref="O22" r:id="rId18"/>
+    <hyperlink ref="O27" r:id="rId19"/>
+    <hyperlink ref="O26" r:id="rId20"/>
+    <hyperlink ref="O25" r:id="rId21"/>
+    <hyperlink ref="O28" r:id="rId22"/>
+    <hyperlink ref="O29" r:id="rId23"/>
+    <hyperlink ref="O30" r:id="rId24"/>
+    <hyperlink ref="O31" r:id="rId25"/>
+    <hyperlink ref="O32" r:id="rId26"/>
+    <hyperlink ref="O34" r:id="rId27"/>
+    <hyperlink ref="O38" r:id="rId28"/>
+    <hyperlink ref="O33" r:id="rId29"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId30"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
#32 IOT Button eSpark BOM 5,100,500 and 5000 updated.
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.3/BOM/eSpark BOM IoT-Button v1.3.xlsx
+++ b/Design Files/IoT-Button-v1.3/BOM/eSpark BOM IoT-Button v1.3.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="207">
   <si>
     <t>Component list</t>
   </si>
@@ -619,6 +619,30 @@
   </si>
   <si>
     <t>Total Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t>Quantity (500 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (500 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (500 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (500 Boards)</t>
+  </si>
+  <si>
+    <t>Quantity (5000 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (5000 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (5000 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (5000 Boards)</t>
   </si>
 </sst>
 </file>
@@ -1075,7 +1099,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1292,6 +1316,9 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1412,6 +1439,114 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="20888325" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19107150" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18916650" y="620017"/>
           <a:ext cx="1714500" cy="1104008"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3572,8 +3707,7 @@
         <v>3</v>
       </c>
       <c r="Q38" s="60">
-        <f t="shared" si="2"/>
-        <v>300</v>
+        <v>3</v>
       </c>
       <c r="R38" s="65" t="s">
         <v>194</v>
@@ -3607,7 +3741,7 @@
       <c r="P39" s="77"/>
       <c r="Q39" s="47">
         <f>SUM(Q10:Q38)</f>
-        <v>384.97899999999998</v>
+        <v>87.978999999999999</v>
       </c>
       <c r="R39" s="72"/>
       <c r="S39" s="73"/>
@@ -3633,7 +3767,7 @@
       <c r="P40" s="77"/>
       <c r="Q40" s="48">
         <f>Q39/5</f>
-        <v>76.995800000000003</v>
+        <v>17.595800000000001</v>
       </c>
       <c r="R40" s="74"/>
       <c r="S40" s="75"/>
@@ -4660,7 +4794,7 @@
         <v>100</v>
       </c>
       <c r="N22" s="37">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="O22" s="59" t="s">
         <v>179</v>
@@ -4670,7 +4804,7 @@
       </c>
       <c r="Q22" s="60">
         <f t="shared" si="2"/>
-        <v>0.68199999999999994</v>
+        <v>4.0919999999999996</v>
       </c>
       <c r="R22" s="37"/>
       <c r="S22" s="58"/>
@@ -4716,7 +4850,7 @@
         <v>100</v>
       </c>
       <c r="N23" s="62">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="O23" s="63" t="s">
         <v>179</v>
@@ -4726,7 +4860,7 @@
       </c>
       <c r="Q23" s="60">
         <f t="shared" si="2"/>
-        <v>0.58799999999999997</v>
+        <v>3.528</v>
       </c>
       <c r="R23" s="50"/>
       <c r="S23" s="58"/>
@@ -4772,7 +4906,7 @@
         <v>700</v>
       </c>
       <c r="N24" s="37">
-        <v>100</v>
+        <v>800</v>
       </c>
       <c r="O24" s="59" t="s">
         <v>179</v>
@@ -4782,7 +4916,7 @@
       </c>
       <c r="Q24" s="60">
         <f t="shared" si="2"/>
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="R24" s="37"/>
       <c r="S24" s="58"/>
@@ -4828,7 +4962,7 @@
         <v>100</v>
       </c>
       <c r="N25" s="37">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="O25" s="59" t="s">
         <v>179</v>
@@ -4838,7 +4972,7 @@
       </c>
       <c r="Q25" s="60">
         <f t="shared" si="2"/>
-        <v>6.9999999999999993E-2</v>
+        <v>0.13999999999999999</v>
       </c>
       <c r="R25" s="50"/>
       <c r="S25" s="58"/>
@@ -4884,7 +5018,7 @@
         <v>200</v>
       </c>
       <c r="N26" s="37">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="O26" s="59" t="s">
         <v>179</v>
@@ -4894,7 +5028,7 @@
       </c>
       <c r="Q26" s="60">
         <f t="shared" si="2"/>
-        <v>0.11</v>
+        <v>0.33</v>
       </c>
       <c r="R26" s="37"/>
       <c r="S26" s="58"/>
@@ -4940,17 +5074,17 @@
         <v>100</v>
       </c>
       <c r="N27" s="37">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="O27" s="59" t="s">
         <v>179</v>
       </c>
       <c r="P27" s="38">
-        <v>1E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="Q27" s="60">
         <f t="shared" si="2"/>
-        <v>0.1</v>
+        <v>0.22</v>
       </c>
       <c r="R27" s="50"/>
       <c r="S27" s="58"/>
@@ -4996,7 +5130,7 @@
         <v>100</v>
       </c>
       <c r="N28" s="37">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="O28" s="59" t="s">
         <v>179</v>
@@ -5006,7 +5140,7 @@
       </c>
       <c r="Q28" s="60">
         <f t="shared" si="2"/>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="R28" s="37"/>
       <c r="S28" s="58"/>
@@ -5052,7 +5186,7 @@
         <v>200</v>
       </c>
       <c r="N29" s="50">
-        <v>20</v>
+        <v>210</v>
       </c>
       <c r="O29" s="61" t="s">
         <v>179</v>
@@ -5062,7 +5196,7 @@
       </c>
       <c r="Q29" s="60">
         <f t="shared" si="2"/>
-        <v>0.79799999999999993</v>
+        <v>8.3789999999999996</v>
       </c>
       <c r="R29" s="50"/>
       <c r="S29" s="58"/>
@@ -5108,17 +5242,17 @@
         <v>100</v>
       </c>
       <c r="N30" s="37">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="O30" s="59" t="s">
         <v>179</v>
       </c>
       <c r="P30" s="38">
-        <v>5.6800000000000003E-2</v>
+        <v>4.5600000000000002E-2</v>
       </c>
       <c r="Q30" s="60">
         <f t="shared" si="2"/>
-        <v>0.56800000000000006</v>
+        <v>5.016</v>
       </c>
       <c r="R30" s="37"/>
       <c r="S30" s="58"/>
@@ -5164,17 +5298,17 @@
         <v>100</v>
       </c>
       <c r="N31" s="37">
-        <v>10</v>
+        <v>105</v>
       </c>
       <c r="O31" s="59" t="s">
         <v>179</v>
       </c>
       <c r="P31" s="38">
-        <v>0.13020000000000001</v>
+        <v>0.1047</v>
       </c>
       <c r="Q31" s="60">
         <f t="shared" si="2"/>
-        <v>1.302</v>
+        <v>10.993500000000001</v>
       </c>
       <c r="R31" s="50"/>
       <c r="S31" s="58"/>
@@ -5220,17 +5354,17 @@
         <v>100</v>
       </c>
       <c r="N32" s="50">
-        <v>10</v>
+        <v>105</v>
       </c>
       <c r="O32" s="61" t="s">
         <v>179</v>
       </c>
       <c r="P32" s="51">
-        <v>0.17599999999999999</v>
+        <v>0.14280000000000001</v>
       </c>
       <c r="Q32" s="60">
         <f t="shared" si="2"/>
-        <v>1.7599999999999998</v>
+        <v>14.994000000000002</v>
       </c>
       <c r="R32" s="37"/>
       <c r="S32" s="58"/>
@@ -5276,7 +5410,7 @@
         <v>100</v>
       </c>
       <c r="N33" s="50">
-        <v>6</v>
+        <v>101</v>
       </c>
       <c r="O33" s="61" t="s">
         <v>179</v>
@@ -5286,7 +5420,7 @@
       </c>
       <c r="Q33" s="60">
         <f t="shared" si="2"/>
-        <v>19.844999999999999</v>
+        <v>334.0575</v>
       </c>
       <c r="R33" s="50"/>
       <c r="S33" s="58"/>
@@ -5332,17 +5466,17 @@
         <v>100</v>
       </c>
       <c r="N34" s="50">
-        <v>6</v>
+        <v>101</v>
       </c>
       <c r="O34" s="61" t="s">
         <v>179</v>
       </c>
       <c r="P34" s="51">
-        <v>0.54569999999999996</v>
+        <v>0.36599999999999999</v>
       </c>
       <c r="Q34" s="60">
         <f t="shared" si="2"/>
-        <v>3.2741999999999996</v>
+        <v>36.966000000000001</v>
       </c>
       <c r="R34" s="37"/>
       <c r="S34" s="58"/>
@@ -5388,7 +5522,7 @@
         <v>100</v>
       </c>
       <c r="N35" s="37">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="O35" s="59" t="s">
         <v>184</v>
@@ -5398,7 +5532,7 @@
       </c>
       <c r="Q35" s="60">
         <f t="shared" si="2"/>
-        <v>23.35</v>
+        <v>467</v>
       </c>
       <c r="R35" s="37"/>
       <c r="S35" s="58"/>
@@ -5556,7 +5690,7 @@
         <v>400</v>
       </c>
       <c r="N38" s="37">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="O38" s="59" t="s">
         <v>184</v>
@@ -5565,8 +5699,7 @@
         <v>3</v>
       </c>
       <c r="Q38" s="60">
-        <f t="shared" si="2"/>
-        <v>300</v>
+        <v>12</v>
       </c>
       <c r="R38" s="65" t="s">
         <v>194</v>
@@ -5594,7 +5727,7 @@
       <c r="P39" s="77"/>
       <c r="Q39" s="47">
         <f>SUM(Q10:Q38)</f>
-        <v>519.67179999999996</v>
+        <v>1065.7405999999999</v>
       </c>
       <c r="R39" s="72"/>
       <c r="S39" s="73"/>
@@ -5620,7 +5753,7 @@
       <c r="P40" s="77"/>
       <c r="Q40" s="48">
         <f>Q39/100</f>
-        <v>5.1967179999999997</v>
+        <v>10.657405999999998</v>
       </c>
       <c r="R40" s="74"/>
       <c r="S40" s="75"/>
@@ -5671,18 +5804,3972 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="68"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="69"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="54" t="s">
+        <v>168</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="70"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="56" t="s">
+        <v>169</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="71"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="57" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="71"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="71"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="71"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="71"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>135</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>199</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>202</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="66"/>
+      <c r="B10" s="45">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I10" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="L10" s="37">
+        <v>6</v>
+      </c>
+      <c r="M10" s="37">
+        <f>L10*500</f>
+        <v>3000</v>
+      </c>
+      <c r="N10" s="37">
+        <v>3100</v>
+      </c>
+      <c r="O10" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P10" s="38">
+        <v>4.7999999999999996E-3</v>
+      </c>
+      <c r="Q10" s="60">
+        <f>P10*N10</f>
+        <v>14.879999999999999</v>
+      </c>
+      <c r="R10" s="37"/>
+      <c r="S10" s="78"/>
+    </row>
+    <row r="11" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A11" s="66"/>
+      <c r="B11" s="46">
+        <f t="shared" ref="B11:B33" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" s="50" t="s">
+        <v>98</v>
+      </c>
+      <c r="H11" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I11" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="J11" s="50" t="s">
+        <v>137</v>
+      </c>
+      <c r="K11" s="50" t="s">
+        <v>160</v>
+      </c>
+      <c r="L11" s="50">
+        <v>15</v>
+      </c>
+      <c r="M11" s="37">
+        <f t="shared" ref="M11:M38" si="1">L11*500</f>
+        <v>7500</v>
+      </c>
+      <c r="N11" s="37">
+        <v>7600</v>
+      </c>
+      <c r="O11" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P11" s="38">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="Q11" s="60">
+        <f t="shared" ref="Q11:Q38" si="2">P11*N11</f>
+        <v>9.879999999999999</v>
+      </c>
+      <c r="R11" s="50"/>
+      <c r="S11" s="50"/>
+    </row>
+    <row r="12" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="66"/>
+      <c r="B12" s="45">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J12" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="K12" s="37" t="s">
+        <v>161</v>
+      </c>
+      <c r="L12" s="37">
+        <v>2</v>
+      </c>
+      <c r="M12" s="37">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N12" s="37">
+        <v>1005</v>
+      </c>
+      <c r="O12" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P12" s="38">
+        <v>9.3200000000000005E-2</v>
+      </c>
+      <c r="Q12" s="60">
+        <f t="shared" si="2"/>
+        <v>93.666000000000011</v>
+      </c>
+      <c r="R12" s="37"/>
+      <c r="S12" s="58"/>
+    </row>
+    <row r="13" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A13" s="66"/>
+      <c r="B13" s="46">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" s="50" t="s">
+        <v>100</v>
+      </c>
+      <c r="H13" s="50" t="s">
+        <v>118</v>
+      </c>
+      <c r="I13" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J13" s="50" t="s">
+        <v>139</v>
+      </c>
+      <c r="K13" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L13" s="50">
+        <v>1</v>
+      </c>
+      <c r="M13" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N13" s="37">
+        <v>510</v>
+      </c>
+      <c r="O13" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P13" s="38">
+        <v>2.41E-2</v>
+      </c>
+      <c r="Q13" s="60">
+        <f t="shared" si="2"/>
+        <v>12.291</v>
+      </c>
+      <c r="R13" s="50"/>
+      <c r="S13" s="58"/>
+    </row>
+    <row r="14" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A14" s="66"/>
+      <c r="B14" s="45">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="K14" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="L14" s="37">
+        <v>1</v>
+      </c>
+      <c r="M14" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N14" s="50">
+        <v>501</v>
+      </c>
+      <c r="O14" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P14" s="51">
+        <v>0.53139999999999998</v>
+      </c>
+      <c r="Q14" s="60">
+        <f t="shared" si="2"/>
+        <v>266.23140000000001</v>
+      </c>
+      <c r="R14" s="37"/>
+      <c r="S14" s="58"/>
+    </row>
+    <row r="15" spans="1:19" s="67" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A15" s="66"/>
+      <c r="B15" s="46">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="53" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="50" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="50" t="s">
+        <v>102</v>
+      </c>
+      <c r="H15" s="50" t="s">
+        <v>120</v>
+      </c>
+      <c r="I15" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J15" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="K15" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L15" s="50">
+        <v>1</v>
+      </c>
+      <c r="M15" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N15" s="37">
+        <v>505</v>
+      </c>
+      <c r="O15" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P15" s="38">
+        <v>6.08E-2</v>
+      </c>
+      <c r="Q15" s="60">
+        <f t="shared" si="2"/>
+        <v>30.704000000000001</v>
+      </c>
+      <c r="R15" s="50"/>
+      <c r="S15" s="58"/>
+    </row>
+    <row r="16" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A16" s="66"/>
+      <c r="B16" s="45">
+        <f>ROW(B16) - ROW($B$9)</f>
+        <v>7</v>
+      </c>
+      <c r="C16" s="52" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="H16" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="I16" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J16" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="K16" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L16" s="37">
+        <v>1</v>
+      </c>
+      <c r="M16" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N16" s="50">
+        <v>520</v>
+      </c>
+      <c r="O16" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P16" s="51">
+        <v>2.07E-2</v>
+      </c>
+      <c r="Q16" s="60">
+        <f t="shared" si="2"/>
+        <v>10.763999999999999</v>
+      </c>
+      <c r="R16" s="37"/>
+      <c r="S16" s="58"/>
+    </row>
+    <row r="17" spans="1:19" s="67" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A17" s="66"/>
+      <c r="B17" s="46">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="C17" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G17" s="50" t="s">
+        <v>82</v>
+      </c>
+      <c r="H17" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="I17" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J17" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="K17" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L17" s="50">
+        <v>1</v>
+      </c>
+      <c r="M17" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N17" s="50">
+        <v>505</v>
+      </c>
+      <c r="O17" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P17" s="38">
+        <v>7.7799999999999994E-2</v>
+      </c>
+      <c r="Q17" s="60">
+        <f t="shared" si="2"/>
+        <v>39.288999999999994</v>
+      </c>
+      <c r="R17" s="50"/>
+      <c r="S17" s="58"/>
+    </row>
+    <row r="18" spans="1:19" s="67" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="66"/>
+      <c r="B18" s="45">
+        <f>ROW(B18) - ROW($B$9)</f>
+        <v>9</v>
+      </c>
+      <c r="C18" s="52" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G18" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J18" s="37" t="s">
+        <v>144</v>
+      </c>
+      <c r="K18" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L18" s="37">
+        <v>1</v>
+      </c>
+      <c r="M18" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N18" s="50">
+        <v>520</v>
+      </c>
+      <c r="O18" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P18" s="51">
+        <v>1.7299999999999999E-2</v>
+      </c>
+      <c r="Q18" s="60">
+        <f t="shared" si="2"/>
+        <v>8.9960000000000004</v>
+      </c>
+      <c r="R18" s="37"/>
+      <c r="S18" s="58"/>
+    </row>
+    <row r="19" spans="1:19" s="67" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A19" s="66"/>
+      <c r="B19" s="46">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C19" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="50" t="s">
+        <v>59</v>
+      </c>
+      <c r="F19" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G19" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="H19" s="50" t="s">
+        <v>124</v>
+      </c>
+      <c r="I19" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J19" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="K19" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L19" s="50">
+        <v>1</v>
+      </c>
+      <c r="M19" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N19" s="37">
+        <v>504</v>
+      </c>
+      <c r="O19" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P19" s="38">
+        <v>4.7300000000000002E-2</v>
+      </c>
+      <c r="Q19" s="60">
+        <f t="shared" si="2"/>
+        <v>23.839200000000002</v>
+      </c>
+      <c r="R19" s="50"/>
+      <c r="S19" s="58"/>
+    </row>
+    <row r="20" spans="1:19" s="67" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A20" s="66"/>
+      <c r="B20" s="45">
+        <f>ROW(B20) - ROW($B$9)</f>
+        <v>11</v>
+      </c>
+      <c r="C20" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="G20" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="H20" s="37" t="s">
+        <v>125</v>
+      </c>
+      <c r="I20" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J20" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="K20" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L20" s="37">
+        <v>1</v>
+      </c>
+      <c r="M20" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N20" s="50">
+        <v>520</v>
+      </c>
+      <c r="O20" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P20" s="51">
+        <v>1.7100000000000001E-2</v>
+      </c>
+      <c r="Q20" s="60">
+        <f t="shared" si="2"/>
+        <v>8.8919999999999995</v>
+      </c>
+      <c r="R20" s="37"/>
+      <c r="S20" s="58"/>
+    </row>
+    <row r="21" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A21" s="66"/>
+      <c r="B21" s="46">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C21" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="50" t="s">
+        <v>35</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G21" s="50" t="s">
+        <v>85</v>
+      </c>
+      <c r="H21" s="50" t="s">
+        <v>126</v>
+      </c>
+      <c r="I21" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J21" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="K21" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L21" s="50">
+        <v>6</v>
+      </c>
+      <c r="M21" s="37">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
+      <c r="N21" s="37">
+        <v>3010</v>
+      </c>
+      <c r="O21" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P21" s="38">
+        <v>4.0099999999999997E-2</v>
+      </c>
+      <c r="Q21" s="60">
+        <f t="shared" si="2"/>
+        <v>120.70099999999999</v>
+      </c>
+      <c r="R21" s="50"/>
+      <c r="S21" s="58"/>
+    </row>
+    <row r="22" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="66"/>
+      <c r="B22" s="45">
+        <f>ROW(B22) - ROW($B$9)</f>
+        <v>13</v>
+      </c>
+      <c r="C22" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="F22" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="G22" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="H22" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="I22" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J22" s="37" t="s">
+        <v>147</v>
+      </c>
+      <c r="K22" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L22" s="37">
+        <v>1</v>
+      </c>
+      <c r="M22" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N22" s="37">
+        <v>520</v>
+      </c>
+      <c r="O22" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P22" s="38">
+        <v>2.7699999999999999E-2</v>
+      </c>
+      <c r="Q22" s="60">
+        <f t="shared" si="2"/>
+        <v>14.404</v>
+      </c>
+      <c r="R22" s="37"/>
+      <c r="S22" s="58"/>
+    </row>
+    <row r="23" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A23" s="66"/>
+      <c r="B23" s="46">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C23" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="E23" s="50" t="s">
+        <v>63</v>
+      </c>
+      <c r="F23" s="50" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" s="50" t="s">
+        <v>107</v>
+      </c>
+      <c r="H23" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="I23" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J23" s="50" t="s">
+        <v>148</v>
+      </c>
+      <c r="K23" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L23" s="50">
+        <v>1</v>
+      </c>
+      <c r="M23" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N23" s="37">
+        <v>520</v>
+      </c>
+      <c r="O23" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P23" s="38">
+        <v>2.3199999999999998E-2</v>
+      </c>
+      <c r="Q23" s="60">
+        <f t="shared" si="2"/>
+        <v>12.064</v>
+      </c>
+      <c r="R23" s="50"/>
+      <c r="S23" s="58"/>
+    </row>
+    <row r="24" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A24" s="66"/>
+      <c r="B24" s="45">
+        <f>ROW(B24) - ROW($B$9)</f>
+        <v>15</v>
+      </c>
+      <c r="C24" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="F24" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G24" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="H24" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I24" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J24" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="K24" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="L24" s="37">
+        <v>7</v>
+      </c>
+      <c r="M24" s="37">
+        <f t="shared" si="1"/>
+        <v>3500</v>
+      </c>
+      <c r="N24" s="37">
+        <v>3600</v>
+      </c>
+      <c r="O24" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P24" s="38">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="Q24" s="60">
+        <f t="shared" si="2"/>
+        <v>2.8800000000000003</v>
+      </c>
+      <c r="R24" s="37"/>
+      <c r="S24" s="58"/>
+    </row>
+    <row r="25" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="66"/>
+      <c r="B25" s="46">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C25" s="53" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="F25" s="50" t="s">
+        <v>89</v>
+      </c>
+      <c r="G25" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="H25" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I25" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J25" s="50" t="s">
+        <v>150</v>
+      </c>
+      <c r="K25" s="50" t="s">
+        <v>163</v>
+      </c>
+      <c r="L25" s="50">
+        <v>1</v>
+      </c>
+      <c r="M25" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N25" s="37">
+        <v>600</v>
+      </c>
+      <c r="O25" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P25" s="38">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q25" s="60">
+        <f t="shared" si="2"/>
+        <v>0.42</v>
+      </c>
+      <c r="R25" s="50"/>
+      <c r="S25" s="58"/>
+    </row>
+    <row r="26" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="66"/>
+      <c r="B26" s="45">
+        <f>ROW(B26) - ROW($B$9)</f>
+        <v>17</v>
+      </c>
+      <c r="C26" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="F26" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G26" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="H26" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I26" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J26" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="K26" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="L26" s="37">
+        <v>2</v>
+      </c>
+      <c r="M26" s="37">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N26" s="37">
+        <v>1100</v>
+      </c>
+      <c r="O26" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P26" s="38">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="Q26" s="60">
+        <f t="shared" si="2"/>
+        <v>0.88</v>
+      </c>
+      <c r="R26" s="37"/>
+      <c r="S26" s="58"/>
+    </row>
+    <row r="27" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="66"/>
+      <c r="B27" s="46">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="C27" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="50" t="s">
+        <v>41</v>
+      </c>
+      <c r="E27" s="50" t="s">
+        <v>67</v>
+      </c>
+      <c r="F27" s="50" t="s">
+        <v>88</v>
+      </c>
+      <c r="G27" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="H27" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I27" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J27" s="50" t="s">
+        <v>152</v>
+      </c>
+      <c r="K27" s="50" t="s">
+        <v>165</v>
+      </c>
+      <c r="L27" s="50">
+        <v>1</v>
+      </c>
+      <c r="M27" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N27" s="37">
+        <v>600</v>
+      </c>
+      <c r="O27" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P27" s="38">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q27" s="60">
+        <f t="shared" si="2"/>
+        <v>0.66</v>
+      </c>
+      <c r="R27" s="50"/>
+      <c r="S27" s="58"/>
+    </row>
+    <row r="28" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A28" s="66"/>
+      <c r="B28" s="45">
+        <f>ROW(B28) - ROW($B$9)</f>
+        <v>19</v>
+      </c>
+      <c r="C28" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="F28" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G28" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="H28" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I28" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J28" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="K28" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="L28" s="37">
+        <v>1</v>
+      </c>
+      <c r="M28" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N28" s="37">
+        <v>600</v>
+      </c>
+      <c r="O28" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P28" s="38">
+        <v>1E-3</v>
+      </c>
+      <c r="Q28" s="60">
+        <f t="shared" si="2"/>
+        <v>0.6</v>
+      </c>
+      <c r="R28" s="37"/>
+      <c r="S28" s="58"/>
+    </row>
+    <row r="29" spans="1:19" s="67" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A29" s="66"/>
+      <c r="B29" s="46">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="C29" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" s="50" t="s">
+        <v>69</v>
+      </c>
+      <c r="F29" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G29" s="50" t="s">
+        <v>90</v>
+      </c>
+      <c r="H29" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="I29" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J29" s="50" t="s">
+        <v>154</v>
+      </c>
+      <c r="K29" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L29" s="50">
+        <v>2</v>
+      </c>
+      <c r="M29" s="37">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N29" s="50">
+        <v>1010</v>
+      </c>
+      <c r="O29" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P29" s="51">
+        <v>2.6800000000000001E-2</v>
+      </c>
+      <c r="Q29" s="60">
+        <f t="shared" si="2"/>
+        <v>27.068000000000001</v>
+      </c>
+      <c r="R29" s="50"/>
+      <c r="S29" s="58"/>
+    </row>
+    <row r="30" spans="1:19" s="67" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A30" s="66"/>
+      <c r="B30" s="45">
+        <f>ROW(B30) - ROW($B$9)</f>
+        <v>21</v>
+      </c>
+      <c r="C30" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G30" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="H30" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="I30" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J30" s="37" t="s">
+        <v>155</v>
+      </c>
+      <c r="K30" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L30" s="37">
+        <v>1</v>
+      </c>
+      <c r="M30" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N30" s="37">
+        <v>510</v>
+      </c>
+      <c r="O30" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P30" s="38">
+        <v>0.04</v>
+      </c>
+      <c r="Q30" s="60">
+        <f t="shared" si="2"/>
+        <v>20.400000000000002</v>
+      </c>
+      <c r="R30" s="37"/>
+      <c r="S30" s="58"/>
+    </row>
+    <row r="31" spans="1:19" s="67" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="66"/>
+      <c r="B31" s="46">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C31" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="F31" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G31" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="H31" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="I31" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J31" s="37" t="s">
+        <v>191</v>
+      </c>
+      <c r="K31" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L31" s="50">
+        <v>1</v>
+      </c>
+      <c r="M31" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N31" s="37">
+        <v>505</v>
+      </c>
+      <c r="O31" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P31" s="38">
+        <v>9.1999999999999998E-2</v>
+      </c>
+      <c r="Q31" s="60">
+        <f t="shared" si="2"/>
+        <v>46.46</v>
+      </c>
+      <c r="R31" s="50"/>
+      <c r="S31" s="58"/>
+    </row>
+    <row r="32" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A32" s="66"/>
+      <c r="B32" s="45">
+        <f>ROW(B32) - ROW($B$9)</f>
+        <v>23</v>
+      </c>
+      <c r="C32" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="F32" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="G32" s="37" t="s">
+        <v>113</v>
+      </c>
+      <c r="H32" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="I32" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J32" s="37" t="s">
+        <v>156</v>
+      </c>
+      <c r="K32" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L32" s="37">
+        <v>1</v>
+      </c>
+      <c r="M32" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N32" s="50">
+        <v>505</v>
+      </c>
+      <c r="O32" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P32" s="51">
+        <v>0.11210000000000001</v>
+      </c>
+      <c r="Q32" s="60">
+        <f t="shared" si="2"/>
+        <v>56.610500000000002</v>
+      </c>
+      <c r="R32" s="37"/>
+      <c r="S32" s="58"/>
+    </row>
+    <row r="33" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A33" s="66"/>
+      <c r="B33" s="46">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="C33" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="E33" s="50" t="s">
+        <v>73</v>
+      </c>
+      <c r="F33" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="G33" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="H33" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="I33" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J33" s="50" t="s">
+        <v>157</v>
+      </c>
+      <c r="K33" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L33" s="50">
+        <v>1</v>
+      </c>
+      <c r="M33" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N33" s="50">
+        <v>501</v>
+      </c>
+      <c r="O33" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P33" s="51">
+        <v>3.3075000000000001</v>
+      </c>
+      <c r="Q33" s="60">
+        <f t="shared" si="2"/>
+        <v>1657.0575000000001</v>
+      </c>
+      <c r="R33" s="50"/>
+      <c r="S33" s="58"/>
+    </row>
+    <row r="34" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A34" s="66"/>
+      <c r="B34" s="45">
+        <f>ROW(B34) - ROW($B$9)</f>
+        <v>25</v>
+      </c>
+      <c r="C34" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>74</v>
+      </c>
+      <c r="F34" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="G34" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="H34" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="I34" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J34" s="37" t="s">
+        <v>158</v>
+      </c>
+      <c r="K34" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L34" s="37">
+        <v>1</v>
+      </c>
+      <c r="M34" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N34" s="50">
+        <v>501</v>
+      </c>
+      <c r="O34" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P34" s="51">
+        <v>0.35160000000000002</v>
+      </c>
+      <c r="Q34" s="60">
+        <f t="shared" si="2"/>
+        <v>176.1516</v>
+      </c>
+      <c r="R34" s="37"/>
+      <c r="S34" s="58"/>
+    </row>
+    <row r="35" spans="1:19" s="67" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A35" s="66"/>
+      <c r="B35" s="45">
+        <f t="shared" ref="B35:B38" si="3">ROW(B35) - ROW($B$9)</f>
+        <v>26</v>
+      </c>
+      <c r="C35" s="52" t="s">
+        <v>181</v>
+      </c>
+      <c r="D35" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E35" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="F35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K35" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L35" s="37">
+        <v>1</v>
+      </c>
+      <c r="M35" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N35" s="37">
+        <v>500</v>
+      </c>
+      <c r="O35" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="P35" s="38">
+        <v>4.67</v>
+      </c>
+      <c r="Q35" s="60">
+        <f t="shared" si="2"/>
+        <v>2335</v>
+      </c>
+      <c r="R35" s="37"/>
+      <c r="S35" s="58"/>
+    </row>
+    <row r="36" spans="1:19" s="67" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A36" s="66"/>
+      <c r="B36" s="45">
+        <f t="shared" si="3"/>
+        <v>27</v>
+      </c>
+      <c r="C36" s="52" t="s">
+        <v>185</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="F36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K36" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L36" s="37">
+        <v>1</v>
+      </c>
+      <c r="M36" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N36" s="37">
+        <v>1</v>
+      </c>
+      <c r="O36" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="P36" s="38">
+        <v>0.35</v>
+      </c>
+      <c r="Q36" s="60">
+        <f t="shared" si="2"/>
+        <v>0.35</v>
+      </c>
+      <c r="R36" s="37"/>
+      <c r="S36" s="58"/>
+    </row>
+    <row r="37" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A37" s="66"/>
+      <c r="B37" s="45">
+        <f t="shared" si="3"/>
+        <v>28</v>
+      </c>
+      <c r="C37" s="52" t="s">
+        <v>187</v>
+      </c>
+      <c r="D37" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E37" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="F37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K37" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L37" s="37">
+        <v>1</v>
+      </c>
+      <c r="M37" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N37" s="37">
+        <v>1</v>
+      </c>
+      <c r="O37" s="59" t="s">
+        <v>188</v>
+      </c>
+      <c r="P37" s="38">
+        <v>16.989999999999998</v>
+      </c>
+      <c r="Q37" s="60">
+        <f t="shared" si="2"/>
+        <v>16.989999999999998</v>
+      </c>
+      <c r="R37" s="37"/>
+      <c r="S37" s="58"/>
+    </row>
+    <row r="38" spans="1:19" s="67" customFormat="1" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="66"/>
+      <c r="B38" s="45">
+        <f t="shared" si="3"/>
+        <v>29</v>
+      </c>
+      <c r="C38" s="52" t="s">
+        <v>192</v>
+      </c>
+      <c r="D38" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E38" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="F38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K38" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L38" s="37">
+        <v>4</v>
+      </c>
+      <c r="M38" s="37">
+        <f t="shared" si="1"/>
+        <v>2000</v>
+      </c>
+      <c r="N38" s="37">
+        <v>2000</v>
+      </c>
+      <c r="O38" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="P38" s="38">
+        <v>3</v>
+      </c>
+      <c r="Q38" s="60">
+        <v>60</v>
+      </c>
+      <c r="R38" s="65" t="s">
+        <v>194</v>
+      </c>
+      <c r="S38" s="58"/>
+    </row>
+    <row r="39" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1"/>
+      <c r="B39" s="39"/>
+      <c r="C39" s="40"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="42"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="44"/>
+      <c r="H39" s="43"/>
+      <c r="I39" s="44"/>
+      <c r="J39" s="43"/>
+      <c r="K39" s="44"/>
+      <c r="L39" s="44"/>
+      <c r="M39" s="44"/>
+      <c r="N39" s="76" t="s">
+        <v>5</v>
+      </c>
+      <c r="O39" s="77"/>
+      <c r="P39" s="77"/>
+      <c r="Q39" s="47">
+        <f>SUM(Q10:Q38)</f>
+        <v>5068.1292000000003</v>
+      </c>
+      <c r="R39" s="72"/>
+      <c r="S39" s="73"/>
+    </row>
+    <row r="40" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="1"/>
+      <c r="B40" s="25"/>
+      <c r="C40" s="36"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="76" t="s">
+        <v>6</v>
+      </c>
+      <c r="O40" s="77"/>
+      <c r="P40" s="77"/>
+      <c r="Q40" s="48">
+        <f>Q39/500</f>
+        <v>10.136258400000001</v>
+      </c>
+      <c r="R40" s="74"/>
+      <c r="S40" s="75"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N39:P39"/>
+    <mergeCell ref="R39:S40"/>
+    <mergeCell ref="N40:P40"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O11" r:id="rId1"/>
+    <hyperlink ref="O35" r:id="rId2"/>
+    <hyperlink ref="O36" r:id="rId3"/>
+    <hyperlink ref="O37" r:id="rId4"/>
+    <hyperlink ref="O10" r:id="rId5"/>
+    <hyperlink ref="O12" r:id="rId6"/>
+    <hyperlink ref="O13" r:id="rId7"/>
+    <hyperlink ref="O15" r:id="rId8"/>
+    <hyperlink ref="O16" r:id="rId9"/>
+    <hyperlink ref="O18" r:id="rId10"/>
+    <hyperlink ref="O19" r:id="rId11"/>
+    <hyperlink ref="O14" r:id="rId12"/>
+    <hyperlink ref="O17" r:id="rId13"/>
+    <hyperlink ref="O20" r:id="rId14"/>
+    <hyperlink ref="O24" r:id="rId15"/>
+    <hyperlink ref="O21" r:id="rId16"/>
+    <hyperlink ref="O23" r:id="rId17"/>
+    <hyperlink ref="O22" r:id="rId18"/>
+    <hyperlink ref="O27" r:id="rId19"/>
+    <hyperlink ref="O26" r:id="rId20"/>
+    <hyperlink ref="O25" r:id="rId21"/>
+    <hyperlink ref="O28" r:id="rId22"/>
+    <hyperlink ref="O29" r:id="rId23"/>
+    <hyperlink ref="O30" r:id="rId24"/>
+    <hyperlink ref="O31" r:id="rId25"/>
+    <hyperlink ref="O32" r:id="rId26"/>
+    <hyperlink ref="O34" r:id="rId27"/>
+    <hyperlink ref="O38" r:id="rId28"/>
+    <hyperlink ref="O33" r:id="rId29"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId30"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="68"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="69"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="54" t="s">
+        <v>168</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="70"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="56" t="s">
+        <v>169</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="71"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="57" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="71"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="71"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="71"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="71"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>135</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>203</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>204</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>206</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="66"/>
+      <c r="B10" s="45">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I10" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="L10" s="37">
+        <v>6</v>
+      </c>
+      <c r="M10" s="37">
+        <f>L10*5000</f>
+        <v>30000</v>
+      </c>
+      <c r="N10" s="37">
+        <v>30100</v>
+      </c>
+      <c r="O10" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P10" s="38">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="Q10" s="60">
+        <f>P10*N10</f>
+        <v>105.35000000000001</v>
+      </c>
+      <c r="R10" s="37"/>
+      <c r="S10" s="78"/>
+    </row>
+    <row r="11" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A11" s="66"/>
+      <c r="B11" s="46">
+        <f t="shared" ref="B11:B33" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" s="50" t="s">
+        <v>98</v>
+      </c>
+      <c r="H11" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I11" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="J11" s="50" t="s">
+        <v>137</v>
+      </c>
+      <c r="K11" s="50" t="s">
+        <v>160</v>
+      </c>
+      <c r="L11" s="50">
+        <v>15</v>
+      </c>
+      <c r="M11" s="37">
+        <f t="shared" ref="M11:M38" si="1">L11*5000</f>
+        <v>75000</v>
+      </c>
+      <c r="N11" s="37">
+        <v>75100</v>
+      </c>
+      <c r="O11" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P11" s="38">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q11" s="60">
+        <f t="shared" ref="Q11:Q38" si="2">P11*N11</f>
+        <v>82.61</v>
+      </c>
+      <c r="R11" s="50"/>
+      <c r="S11" s="50"/>
+    </row>
+    <row r="12" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="66"/>
+      <c r="B12" s="45">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J12" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="K12" s="37" t="s">
+        <v>161</v>
+      </c>
+      <c r="L12" s="37">
+        <v>2</v>
+      </c>
+      <c r="M12" s="37">
+        <f t="shared" si="1"/>
+        <v>10000</v>
+      </c>
+      <c r="N12" s="37">
+        <v>10100</v>
+      </c>
+      <c r="O12" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P12" s="38">
+        <v>7.85E-2</v>
+      </c>
+      <c r="Q12" s="60">
+        <f t="shared" si="2"/>
+        <v>792.85</v>
+      </c>
+      <c r="R12" s="37"/>
+      <c r="S12" s="58"/>
+    </row>
+    <row r="13" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="66"/>
+      <c r="B13" s="46">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" s="50" t="s">
+        <v>100</v>
+      </c>
+      <c r="H13" s="50" t="s">
+        <v>118</v>
+      </c>
+      <c r="I13" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J13" s="50" t="s">
+        <v>139</v>
+      </c>
+      <c r="K13" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L13" s="50">
+        <v>1</v>
+      </c>
+      <c r="M13" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N13" s="37">
+        <v>5010</v>
+      </c>
+      <c r="O13" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P13" s="38">
+        <v>1.8599999999999998E-2</v>
+      </c>
+      <c r="Q13" s="60">
+        <f t="shared" si="2"/>
+        <v>93.185999999999993</v>
+      </c>
+      <c r="R13" s="50"/>
+      <c r="S13" s="58"/>
+    </row>
+    <row r="14" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A14" s="66"/>
+      <c r="B14" s="45">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="K14" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="L14" s="37">
+        <v>1</v>
+      </c>
+      <c r="M14" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N14" s="50">
+        <v>5001</v>
+      </c>
+      <c r="O14" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P14" s="51">
+        <v>0.51229999999999998</v>
+      </c>
+      <c r="Q14" s="60">
+        <f t="shared" si="2"/>
+        <v>2562.0122999999999</v>
+      </c>
+      <c r="R14" s="37"/>
+      <c r="S14" s="58"/>
+    </row>
+    <row r="15" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A15" s="66"/>
+      <c r="B15" s="46">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="53" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="50" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="50" t="s">
+        <v>102</v>
+      </c>
+      <c r="H15" s="50" t="s">
+        <v>120</v>
+      </c>
+      <c r="I15" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J15" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="K15" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L15" s="50">
+        <v>1</v>
+      </c>
+      <c r="M15" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N15" s="37">
+        <v>5005</v>
+      </c>
+      <c r="O15" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P15" s="38">
+        <v>4.8899999999999999E-2</v>
+      </c>
+      <c r="Q15" s="60">
+        <f t="shared" si="2"/>
+        <v>244.74449999999999</v>
+      </c>
+      <c r="R15" s="50"/>
+      <c r="S15" s="58"/>
+    </row>
+    <row r="16" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A16" s="66"/>
+      <c r="B16" s="45">
+        <f>ROW(B16) - ROW($B$9)</f>
+        <v>7</v>
+      </c>
+      <c r="C16" s="52" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="H16" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="I16" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J16" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="K16" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L16" s="37">
+        <v>1</v>
+      </c>
+      <c r="M16" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N16" s="50">
+        <v>5020</v>
+      </c>
+      <c r="O16" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P16" s="51">
+        <v>1.6299999999999999E-2</v>
+      </c>
+      <c r="Q16" s="60">
+        <f t="shared" si="2"/>
+        <v>81.825999999999993</v>
+      </c>
+      <c r="R16" s="37"/>
+      <c r="S16" s="58"/>
+    </row>
+    <row r="17" spans="1:19" s="67" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A17" s="66"/>
+      <c r="B17" s="46">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="C17" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G17" s="50" t="s">
+        <v>82</v>
+      </c>
+      <c r="H17" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="I17" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J17" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="K17" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L17" s="50">
+        <v>1</v>
+      </c>
+      <c r="M17" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N17" s="50">
+        <v>5005</v>
+      </c>
+      <c r="O17" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P17" s="38">
+        <v>6.7799999999999999E-2</v>
+      </c>
+      <c r="Q17" s="60">
+        <f t="shared" si="2"/>
+        <v>339.339</v>
+      </c>
+      <c r="R17" s="50"/>
+      <c r="S17" s="58"/>
+    </row>
+    <row r="18" spans="1:19" s="67" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A18" s="66"/>
+      <c r="B18" s="45">
+        <f>ROW(B18) - ROW($B$9)</f>
+        <v>9</v>
+      </c>
+      <c r="C18" s="52" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G18" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J18" s="37" t="s">
+        <v>144</v>
+      </c>
+      <c r="K18" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L18" s="37">
+        <v>1</v>
+      </c>
+      <c r="M18" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N18" s="50">
+        <v>5020</v>
+      </c>
+      <c r="O18" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P18" s="51">
+        <v>1.24E-2</v>
+      </c>
+      <c r="Q18" s="60">
+        <f t="shared" si="2"/>
+        <v>62.247999999999998</v>
+      </c>
+      <c r="R18" s="37"/>
+      <c r="S18" s="58"/>
+    </row>
+    <row r="19" spans="1:19" s="67" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A19" s="66"/>
+      <c r="B19" s="46">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C19" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="50" t="s">
+        <v>59</v>
+      </c>
+      <c r="F19" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G19" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="H19" s="50" t="s">
+        <v>124</v>
+      </c>
+      <c r="I19" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J19" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="K19" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L19" s="50">
+        <v>1</v>
+      </c>
+      <c r="M19" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N19" s="37">
+        <v>5004</v>
+      </c>
+      <c r="O19" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P19" s="38">
+        <v>4.2599999999999999E-2</v>
+      </c>
+      <c r="Q19" s="60">
+        <f t="shared" si="2"/>
+        <v>213.1704</v>
+      </c>
+      <c r="R19" s="50"/>
+      <c r="S19" s="58"/>
+    </row>
+    <row r="20" spans="1:19" s="67" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A20" s="66"/>
+      <c r="B20" s="45">
+        <f>ROW(B20) - ROW($B$9)</f>
+        <v>11</v>
+      </c>
+      <c r="C20" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="G20" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="H20" s="37" t="s">
+        <v>125</v>
+      </c>
+      <c r="I20" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J20" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="K20" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L20" s="37">
+        <v>1</v>
+      </c>
+      <c r="M20" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N20" s="50">
+        <v>5020</v>
+      </c>
+      <c r="O20" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P20" s="51">
+        <v>1.3100000000000001E-2</v>
+      </c>
+      <c r="Q20" s="60">
+        <f t="shared" si="2"/>
+        <v>65.762</v>
+      </c>
+      <c r="R20" s="37"/>
+      <c r="S20" s="58"/>
+    </row>
+    <row r="21" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A21" s="66"/>
+      <c r="B21" s="46">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C21" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="50" t="s">
+        <v>35</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G21" s="50" t="s">
+        <v>85</v>
+      </c>
+      <c r="H21" s="50" t="s">
+        <v>126</v>
+      </c>
+      <c r="I21" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J21" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="K21" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L21" s="50">
+        <v>6</v>
+      </c>
+      <c r="M21" s="37">
+        <f t="shared" si="1"/>
+        <v>30000</v>
+      </c>
+      <c r="N21" s="37">
+        <v>30010</v>
+      </c>
+      <c r="O21" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P21" s="38">
+        <v>3.49E-2</v>
+      </c>
+      <c r="Q21" s="60">
+        <f t="shared" si="2"/>
+        <v>1047.3489999999999</v>
+      </c>
+      <c r="R21" s="50"/>
+      <c r="S21" s="58"/>
+    </row>
+    <row r="22" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="66"/>
+      <c r="B22" s="45">
+        <f>ROW(B22) - ROW($B$9)</f>
+        <v>13</v>
+      </c>
+      <c r="C22" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="F22" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="G22" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="H22" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="I22" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J22" s="37" t="s">
+        <v>147</v>
+      </c>
+      <c r="K22" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L22" s="37">
+        <v>1</v>
+      </c>
+      <c r="M22" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N22" s="37">
+        <v>5020</v>
+      </c>
+      <c r="O22" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P22" s="38">
+        <v>1.89E-2</v>
+      </c>
+      <c r="Q22" s="60">
+        <f t="shared" si="2"/>
+        <v>94.878</v>
+      </c>
+      <c r="R22" s="37"/>
+      <c r="S22" s="58"/>
+    </row>
+    <row r="23" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A23" s="66"/>
+      <c r="B23" s="46">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C23" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="E23" s="50" t="s">
+        <v>63</v>
+      </c>
+      <c r="F23" s="50" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" s="50" t="s">
+        <v>107</v>
+      </c>
+      <c r="H23" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="I23" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J23" s="50" t="s">
+        <v>148</v>
+      </c>
+      <c r="K23" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L23" s="50">
+        <v>1</v>
+      </c>
+      <c r="M23" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N23" s="37">
+        <v>5020</v>
+      </c>
+      <c r="O23" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P23" s="38">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="Q23" s="60">
+        <f t="shared" si="2"/>
+        <v>90.36</v>
+      </c>
+      <c r="R23" s="50"/>
+      <c r="S23" s="58"/>
+    </row>
+    <row r="24" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="66"/>
+      <c r="B24" s="45">
+        <f>ROW(B24) - ROW($B$9)</f>
+        <v>15</v>
+      </c>
+      <c r="C24" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="F24" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G24" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="H24" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I24" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J24" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="K24" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="L24" s="37">
+        <v>7</v>
+      </c>
+      <c r="M24" s="37">
+        <f t="shared" si="1"/>
+        <v>35000</v>
+      </c>
+      <c r="N24" s="37">
+        <v>35100</v>
+      </c>
+      <c r="O24" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P24" s="38">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="Q24" s="60">
+        <f t="shared" si="2"/>
+        <v>21.06</v>
+      </c>
+      <c r="R24" s="37"/>
+      <c r="S24" s="58"/>
+    </row>
+    <row r="25" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="66"/>
+      <c r="B25" s="46">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C25" s="53" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="F25" s="50" t="s">
+        <v>89</v>
+      </c>
+      <c r="G25" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="H25" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I25" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J25" s="50" t="s">
+        <v>150</v>
+      </c>
+      <c r="K25" s="50" t="s">
+        <v>163</v>
+      </c>
+      <c r="L25" s="50">
+        <v>1</v>
+      </c>
+      <c r="M25" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N25" s="37">
+        <v>5100</v>
+      </c>
+      <c r="O25" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P25" s="38">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="Q25" s="60">
+        <f t="shared" si="2"/>
+        <v>2.5500000000000003</v>
+      </c>
+      <c r="R25" s="50"/>
+      <c r="S25" s="58"/>
+    </row>
+    <row r="26" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="66"/>
+      <c r="B26" s="45">
+        <f>ROW(B26) - ROW($B$9)</f>
+        <v>17</v>
+      </c>
+      <c r="C26" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="F26" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G26" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="H26" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I26" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J26" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="K26" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="L26" s="37">
+        <v>2</v>
+      </c>
+      <c r="M26" s="37">
+        <f t="shared" si="1"/>
+        <v>10000</v>
+      </c>
+      <c r="N26" s="37">
+        <v>10100</v>
+      </c>
+      <c r="O26" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P26" s="38">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q26" s="60">
+        <f t="shared" si="2"/>
+        <v>7.07</v>
+      </c>
+      <c r="R26" s="37"/>
+      <c r="S26" s="58"/>
+    </row>
+    <row r="27" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="66"/>
+      <c r="B27" s="46">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="C27" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="50" t="s">
+        <v>41</v>
+      </c>
+      <c r="E27" s="50" t="s">
+        <v>67</v>
+      </c>
+      <c r="F27" s="50" t="s">
+        <v>88</v>
+      </c>
+      <c r="G27" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="H27" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I27" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J27" s="50" t="s">
+        <v>152</v>
+      </c>
+      <c r="K27" s="50" t="s">
+        <v>165</v>
+      </c>
+      <c r="L27" s="50">
+        <v>1</v>
+      </c>
+      <c r="M27" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N27" s="37">
+        <v>5100</v>
+      </c>
+      <c r="O27" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P27" s="38">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q27" s="60">
+        <f t="shared" si="2"/>
+        <v>3.57</v>
+      </c>
+      <c r="R27" s="50"/>
+      <c r="S27" s="58"/>
+    </row>
+    <row r="28" spans="1:19" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="66"/>
+      <c r="B28" s="45">
+        <f>ROW(B28) - ROW($B$9)</f>
+        <v>19</v>
+      </c>
+      <c r="C28" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="F28" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G28" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="H28" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="I28" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J28" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="K28" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="L28" s="37">
+        <v>1</v>
+      </c>
+      <c r="M28" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N28" s="37">
+        <v>5100</v>
+      </c>
+      <c r="O28" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P28" s="38">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q28" s="60">
+        <f t="shared" si="2"/>
+        <v>3.57</v>
+      </c>
+      <c r="R28" s="37"/>
+      <c r="S28" s="58"/>
+    </row>
+    <row r="29" spans="1:19" s="67" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A29" s="66"/>
+      <c r="B29" s="46">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="C29" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" s="50" t="s">
+        <v>69</v>
+      </c>
+      <c r="F29" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G29" s="50" t="s">
+        <v>90</v>
+      </c>
+      <c r="H29" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="I29" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J29" s="50" t="s">
+        <v>154</v>
+      </c>
+      <c r="K29" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L29" s="50">
+        <v>2</v>
+      </c>
+      <c r="M29" s="37">
+        <f t="shared" si="1"/>
+        <v>10000</v>
+      </c>
+      <c r="N29" s="50">
+        <v>10010</v>
+      </c>
+      <c r="O29" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P29" s="51">
+        <v>2.3699999999999999E-2</v>
+      </c>
+      <c r="Q29" s="60">
+        <f t="shared" si="2"/>
+        <v>237.23699999999999</v>
+      </c>
+      <c r="R29" s="50"/>
+      <c r="S29" s="58"/>
+    </row>
+    <row r="30" spans="1:19" s="67" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A30" s="66"/>
+      <c r="B30" s="45">
+        <f>ROW(B30) - ROW($B$9)</f>
+        <v>21</v>
+      </c>
+      <c r="C30" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G30" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="H30" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="I30" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J30" s="37" t="s">
+        <v>155</v>
+      </c>
+      <c r="K30" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L30" s="37">
+        <v>1</v>
+      </c>
+      <c r="M30" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N30" s="37">
+        <v>5010</v>
+      </c>
+      <c r="O30" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P30" s="38">
+        <v>3.2399999999999998E-2</v>
+      </c>
+      <c r="Q30" s="60">
+        <f t="shared" si="2"/>
+        <v>162.32399999999998</v>
+      </c>
+      <c r="R30" s="37"/>
+      <c r="S30" s="58"/>
+    </row>
+    <row r="31" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A31" s="66"/>
+      <c r="B31" s="46">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C31" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="F31" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="G31" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="H31" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="I31" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J31" s="37" t="s">
+        <v>191</v>
+      </c>
+      <c r="K31" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L31" s="50">
+        <v>1</v>
+      </c>
+      <c r="M31" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N31" s="37">
+        <v>5005</v>
+      </c>
+      <c r="O31" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="P31" s="38">
+        <v>7.0999999999999994E-2</v>
+      </c>
+      <c r="Q31" s="60">
+        <f t="shared" si="2"/>
+        <v>355.35499999999996</v>
+      </c>
+      <c r="R31" s="50"/>
+      <c r="S31" s="58"/>
+    </row>
+    <row r="32" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A32" s="66"/>
+      <c r="B32" s="45">
+        <f>ROW(B32) - ROW($B$9)</f>
+        <v>23</v>
+      </c>
+      <c r="C32" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="F32" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="G32" s="37" t="s">
+        <v>113</v>
+      </c>
+      <c r="H32" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="I32" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J32" s="37" t="s">
+        <v>156</v>
+      </c>
+      <c r="K32" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L32" s="37">
+        <v>1</v>
+      </c>
+      <c r="M32" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N32" s="50">
+        <v>5005</v>
+      </c>
+      <c r="O32" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P32" s="51">
+        <v>8.9200000000000002E-2</v>
+      </c>
+      <c r="Q32" s="60">
+        <f t="shared" si="2"/>
+        <v>446.44600000000003</v>
+      </c>
+      <c r="R32" s="37"/>
+      <c r="S32" s="58"/>
+    </row>
+    <row r="33" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A33" s="66"/>
+      <c r="B33" s="46">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="C33" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="E33" s="50" t="s">
+        <v>73</v>
+      </c>
+      <c r="F33" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="G33" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="H33" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="I33" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J33" s="50" t="s">
+        <v>157</v>
+      </c>
+      <c r="K33" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L33" s="50">
+        <v>1</v>
+      </c>
+      <c r="M33" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N33" s="50">
+        <v>5001</v>
+      </c>
+      <c r="O33" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P33" s="51">
+        <v>3.3075000000000001</v>
+      </c>
+      <c r="Q33" s="60">
+        <f t="shared" si="2"/>
+        <v>16540.807499999999</v>
+      </c>
+      <c r="R33" s="50"/>
+      <c r="S33" s="58"/>
+    </row>
+    <row r="34" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A34" s="66"/>
+      <c r="B34" s="45">
+        <f>ROW(B34) - ROW($B$9)</f>
+        <v>25</v>
+      </c>
+      <c r="C34" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>74</v>
+      </c>
+      <c r="F34" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="G34" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="H34" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="I34" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J34" s="37" t="s">
+        <v>158</v>
+      </c>
+      <c r="K34" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L34" s="37">
+        <v>1</v>
+      </c>
+      <c r="M34" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N34" s="50">
+        <v>5001</v>
+      </c>
+      <c r="O34" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="P34" s="51">
+        <v>0.34210000000000002</v>
+      </c>
+      <c r="Q34" s="60">
+        <f t="shared" si="2"/>
+        <v>1710.8421000000001</v>
+      </c>
+      <c r="R34" s="37"/>
+      <c r="S34" s="58"/>
+    </row>
+    <row r="35" spans="1:19" s="67" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A35" s="66"/>
+      <c r="B35" s="45">
+        <f t="shared" ref="B35:B38" si="3">ROW(B35) - ROW($B$9)</f>
+        <v>26</v>
+      </c>
+      <c r="C35" s="52" t="s">
+        <v>181</v>
+      </c>
+      <c r="D35" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E35" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="F35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J35" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K35" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L35" s="37">
+        <v>1</v>
+      </c>
+      <c r="M35" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N35" s="37">
+        <v>5000</v>
+      </c>
+      <c r="O35" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="P35" s="38">
+        <v>4.67</v>
+      </c>
+      <c r="Q35" s="60">
+        <f t="shared" si="2"/>
+        <v>23350</v>
+      </c>
+      <c r="R35" s="37"/>
+      <c r="S35" s="58"/>
+    </row>
+    <row r="36" spans="1:19" s="67" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A36" s="66"/>
+      <c r="B36" s="45">
+        <f t="shared" si="3"/>
+        <v>27</v>
+      </c>
+      <c r="C36" s="52" t="s">
+        <v>185</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="F36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J36" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K36" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L36" s="37">
+        <v>1</v>
+      </c>
+      <c r="M36" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N36" s="37">
+        <v>1</v>
+      </c>
+      <c r="O36" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="P36" s="38">
+        <v>0.35</v>
+      </c>
+      <c r="Q36" s="60">
+        <f t="shared" si="2"/>
+        <v>0.35</v>
+      </c>
+      <c r="R36" s="37"/>
+      <c r="S36" s="58"/>
+    </row>
+    <row r="37" spans="1:19" s="67" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A37" s="66"/>
+      <c r="B37" s="45">
+        <f t="shared" si="3"/>
+        <v>28</v>
+      </c>
+      <c r="C37" s="52" t="s">
+        <v>187</v>
+      </c>
+      <c r="D37" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E37" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="F37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J37" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K37" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L37" s="37">
+        <v>1</v>
+      </c>
+      <c r="M37" s="37">
+        <f t="shared" si="1"/>
+        <v>5000</v>
+      </c>
+      <c r="N37" s="37">
+        <v>1</v>
+      </c>
+      <c r="O37" s="59" t="s">
+        <v>188</v>
+      </c>
+      <c r="P37" s="38">
+        <v>16.989999999999998</v>
+      </c>
+      <c r="Q37" s="60">
+        <f t="shared" si="2"/>
+        <v>16.989999999999998</v>
+      </c>
+      <c r="R37" s="37"/>
+      <c r="S37" s="58"/>
+    </row>
+    <row r="38" spans="1:19" s="67" customFormat="1" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="66"/>
+      <c r="B38" s="45">
+        <f t="shared" si="3"/>
+        <v>29</v>
+      </c>
+      <c r="C38" s="52" t="s">
+        <v>192</v>
+      </c>
+      <c r="D38" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="E38" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="F38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="G38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="I38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J38" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="K38" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="L38" s="37">
+        <v>4</v>
+      </c>
+      <c r="M38" s="37">
+        <f t="shared" si="1"/>
+        <v>20000</v>
+      </c>
+      <c r="N38" s="37">
+        <v>20000</v>
+      </c>
+      <c r="O38" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="P38" s="38">
+        <v>3</v>
+      </c>
+      <c r="Q38" s="60">
+        <v>600</v>
+      </c>
+      <c r="R38" s="65" t="s">
+        <v>194</v>
+      </c>
+      <c r="S38" s="58"/>
+    </row>
+    <row r="39" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1"/>
+      <c r="B39" s="39"/>
+      <c r="C39" s="40"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="42"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="44"/>
+      <c r="H39" s="43"/>
+      <c r="I39" s="44"/>
+      <c r="J39" s="43"/>
+      <c r="K39" s="44"/>
+      <c r="L39" s="44"/>
+      <c r="M39" s="44"/>
+      <c r="N39" s="76" t="s">
+        <v>5</v>
+      </c>
+      <c r="O39" s="77"/>
+      <c r="P39" s="77"/>
+      <c r="Q39" s="47">
+        <f>SUM(Q10:Q38)</f>
+        <v>49333.856799999994</v>
+      </c>
+      <c r="R39" s="72"/>
+      <c r="S39" s="73"/>
+    </row>
+    <row r="40" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="1"/>
+      <c r="B40" s="25"/>
+      <c r="C40" s="36"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="76" t="s">
+        <v>6</v>
+      </c>
+      <c r="O40" s="77"/>
+      <c r="P40" s="77"/>
+      <c r="Q40" s="48">
+        <f>Q39/5000</f>
+        <v>9.8667713599999995</v>
+      </c>
+      <c r="R40" s="74"/>
+      <c r="S40" s="75"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N39:P39"/>
+    <mergeCell ref="R39:S40"/>
+    <mergeCell ref="N40:P40"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O11" r:id="rId1"/>
+    <hyperlink ref="O35" r:id="rId2"/>
+    <hyperlink ref="O36" r:id="rId3"/>
+    <hyperlink ref="O37" r:id="rId4"/>
+    <hyperlink ref="O10" r:id="rId5"/>
+    <hyperlink ref="O12" r:id="rId6"/>
+    <hyperlink ref="O13" r:id="rId7"/>
+    <hyperlink ref="O15" r:id="rId8"/>
+    <hyperlink ref="O16" r:id="rId9"/>
+    <hyperlink ref="O18" r:id="rId10"/>
+    <hyperlink ref="O19" r:id="rId11"/>
+    <hyperlink ref="O14" r:id="rId12"/>
+    <hyperlink ref="O17" r:id="rId13"/>
+    <hyperlink ref="O20" r:id="rId14"/>
+    <hyperlink ref="O24" r:id="rId15"/>
+    <hyperlink ref="O21" r:id="rId16"/>
+    <hyperlink ref="O23" r:id="rId17"/>
+    <hyperlink ref="O22" r:id="rId18"/>
+    <hyperlink ref="O27" r:id="rId19"/>
+    <hyperlink ref="O26" r:id="rId20"/>
+    <hyperlink ref="O25" r:id="rId21"/>
+    <hyperlink ref="O28" r:id="rId22"/>
+    <hyperlink ref="O29" r:id="rId23"/>
+    <hyperlink ref="O30" r:id="rId24"/>
+    <hyperlink ref="O31" r:id="rId25"/>
+    <hyperlink ref="O32" r:id="rId26"/>
+    <hyperlink ref="O34" r:id="rId27"/>
+    <hyperlink ref="O38" r:id="rId28"/>
+    <hyperlink ref="O33" r:id="rId29"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId30"/>
 </worksheet>
 </file>
</xml_diff>